<commit_message>
Refresh demo data from latest lowp v14 exports, 10 -> 15 points per line
The lowp exports supersede the earlier high-power runs (base AETOT now
~295 MW, matching the corrected base model). Demo subsets resampled
evenly across the MCH feed-flow range; banner and entry text updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/lohc-dashboard/demo/lohc_demo_line5.xlsx
+++ b/public/lohc-dashboard/demo/lohc_demo_line5.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CF11"/>
+  <dimension ref="A1:CF16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -856,7 +856,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>821.450336</v>
+        <v>810.160655</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -865,64 +865,64 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="J2" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="K2" t="n">
-        <v>19.49</v>
+        <v>15</v>
       </c>
       <c r="L2" t="n">
         <v>1500</v>
       </c>
       <c r="M2" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="N2" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="O2" t="n">
         <v>1.034</v>
       </c>
       <c r="P2" t="n">
-        <v>642.22253</v>
+        <v>701.938526</v>
       </c>
       <c r="Q2" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="R2" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="S2" t="n">
         <v>1.027</v>
       </c>
       <c r="T2" t="n">
-        <v>377.973001</v>
+        <v>437.026285</v>
       </c>
       <c r="U2" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="V2" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="W2" t="n">
         <v>1.02</v>
       </c>
       <c r="X2" t="n">
-        <v>206.058218</v>
+        <v>208.515331</v>
       </c>
       <c r="Y2" t="n">
-        <v>272.860474</v>
+        <v>263.524695</v>
       </c>
       <c r="Z2" t="n">
-        <v>9.67455243</v>
+        <v>9.3509885</v>
       </c>
       <c r="AA2" t="n">
         <v>1.034</v>
       </c>
       <c r="AB2" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AC2" t="n">
         <v>70</v>
@@ -934,70 +934,70 @@
         <v>50</v>
       </c>
       <c r="AF2" t="n">
-        <v>475.214164</v>
+        <v>595.781791</v>
       </c>
       <c r="AG2" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AH2" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AI2" t="n">
         <v>1.013</v>
       </c>
       <c r="AJ2" t="n">
-        <v>191.433655</v>
+        <v>194.807216</v>
       </c>
       <c r="AK2" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AL2" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AM2" t="n">
         <v>1.034</v>
       </c>
       <c r="AN2" t="n">
-        <v>640.328118</v>
+        <v>700.032375</v>
       </c>
       <c r="AO2" t="n">
-        <v>-258041.636</v>
+        <v>-241187.022</v>
       </c>
       <c r="AP2" t="n">
-        <v>-47299.3164</v>
+        <v>-54582.3724</v>
       </c>
       <c r="AQ2" t="n">
         <v>32.9836374</v>
       </c>
       <c r="AR2" t="n">
-        <v>397.974738</v>
+        <v>400.505948</v>
       </c>
       <c r="AS2" t="n">
-        <v>-304909.994</v>
+        <v>-295335.904</v>
       </c>
       <c r="AT2" t="n">
-        <v>84.3022258</v>
+        <v>81.4178692</v>
       </c>
       <c r="AU2" t="n">
-        <v>2.98902326</v>
+        <v>2.88905583</v>
       </c>
       <c r="AV2" t="n">
         <v>1.034</v>
       </c>
       <c r="AW2" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AX2" t="n">
-        <v>84.3022258</v>
+        <v>81.4178692</v>
       </c>
       <c r="AY2" t="n">
-        <v>2.98902326</v>
+        <v>2.88905583</v>
       </c>
       <c r="AZ2" t="n">
         <v>1.034</v>
       </c>
       <c r="BA2" t="n">
-        <v>634.191031</v>
+        <v>693.857862</v>
       </c>
       <c r="BB2" t="n">
         <v>0.302437437</v>
@@ -1021,37 +1021,37 @@
         <v>2.64033899</v>
       </c>
       <c r="BI2" t="n">
-        <v>467.584356</v>
+        <v>515.504448</v>
       </c>
       <c r="BJ2" t="n">
         <v>0.302437437</v>
       </c>
       <c r="BK2" t="n">
-        <v>0.0121419382</v>
+        <v>0.0117611672</v>
       </c>
       <c r="BL2" t="n">
         <v>2.64033899</v>
       </c>
       <c r="BM2" t="n">
-        <v>155.845749</v>
+        <v>176.925852</v>
       </c>
       <c r="BN2" t="n">
-        <v>0.00490836502</v>
+        <v>0.0158590325</v>
       </c>
       <c r="BO2" t="n">
-        <v>0.746318726</v>
+        <v>0.738105726</v>
       </c>
       <c r="BP2" t="n">
         <v>0.302437437</v>
       </c>
       <c r="BQ2" t="n">
-        <v>0.0121419382</v>
+        <v>0.0117611672</v>
       </c>
       <c r="BR2" t="n">
         <v>2.64033899</v>
       </c>
       <c r="BS2" t="n">
-        <v>634.038811</v>
+        <v>693.604565</v>
       </c>
       <c r="BT2" t="n">
         <v>70</v>
@@ -1063,7 +1063,7 @@
         <v>50.07</v>
       </c>
       <c r="BW2" t="n">
-        <v>173.839455</v>
+        <v>179.187081</v>
       </c>
       <c r="BX2" t="n">
         <v>70</v>
@@ -1075,7 +1075,7 @@
         <v>50.05</v>
       </c>
       <c r="CA2" t="n">
-        <v>192.390605</v>
+        <v>195.872202</v>
       </c>
       <c r="CB2" t="n">
         <v>70</v>
@@ -1090,27 +1090,27 @@
         <v>264.0032</v>
       </c>
       <c r="CF2" t="n">
-        <v>12.19</v>
+        <v>12.15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="B3" t="n">
-        <v>0.7352551381053591</v>
+        <v>0.8601227089320744</v>
       </c>
       <c r="C3" t="n">
-        <v>1.358282460385504</v>
+        <v>4.40854338138764</v>
       </c>
       <c r="D3" t="n">
-        <v>5.508552353007732</v>
+        <v>5.039034289413324</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>4615.94757</v>
+        <v>3620.06109</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -1119,64 +1119,64 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="J3" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="K3" t="n">
-        <v>19.49</v>
+        <v>15</v>
       </c>
       <c r="L3" t="n">
         <v>1500</v>
       </c>
       <c r="M3" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="N3" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="O3" t="n">
         <v>1.034</v>
       </c>
       <c r="P3" t="n">
-        <v>642.22253</v>
+        <v>701.938526</v>
       </c>
       <c r="Q3" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="R3" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="S3" t="n">
         <v>1.027</v>
       </c>
       <c r="T3" t="n">
-        <v>368.066465</v>
+        <v>426.933039</v>
       </c>
       <c r="U3" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="V3" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="W3" t="n">
         <v>1.02</v>
       </c>
       <c r="X3" t="n">
-        <v>205.397982</v>
+        <v>207.675526</v>
       </c>
       <c r="Y3" t="n">
-        <v>262.60571</v>
+        <v>296.692933</v>
       </c>
       <c r="Z3" t="n">
-        <v>9.310959090000001</v>
+        <v>10.5279401</v>
       </c>
       <c r="AA3" t="n">
         <v>1.034</v>
       </c>
       <c r="AB3" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AC3" t="n">
         <v>70</v>
@@ -1188,124 +1188,124 @@
         <v>50</v>
       </c>
       <c r="AF3" t="n">
-        <v>452.327153</v>
+        <v>578.94693</v>
       </c>
       <c r="AG3" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AH3" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AI3" t="n">
         <v>1.013</v>
       </c>
       <c r="AJ3" t="n">
-        <v>190.609316</v>
+        <v>194.002151</v>
       </c>
       <c r="AK3" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AL3" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AM3" t="n">
         <v>1.034</v>
       </c>
       <c r="AN3" t="n">
-        <v>631.5670730000001</v>
+        <v>693.415543</v>
       </c>
       <c r="AO3" t="n">
-        <v>-258041.636</v>
+        <v>-241187.022</v>
       </c>
       <c r="AP3" t="n">
-        <v>-45937.8059</v>
+        <v>-53549.8399</v>
       </c>
       <c r="AQ3" t="n">
         <v>32.9836374</v>
       </c>
       <c r="AR3" t="n">
-        <v>397.499704</v>
+        <v>400.146789</v>
       </c>
       <c r="AS3" t="n">
-        <v>-303548.958</v>
+        <v>-294303.731</v>
       </c>
       <c r="AT3" t="n">
-        <v>94.55698959999999</v>
+        <v>48.2496315</v>
       </c>
       <c r="AU3" t="n">
-        <v>3.3526166</v>
+        <v>1.71210424</v>
       </c>
       <c r="AV3" t="n">
         <v>1.034</v>
       </c>
       <c r="AW3" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AX3" t="n">
-        <v>94.55698959999999</v>
+        <v>48.2496315</v>
       </c>
       <c r="AY3" t="n">
-        <v>3.3526166</v>
+        <v>1.71210424</v>
       </c>
       <c r="AZ3" t="n">
         <v>1.034</v>
       </c>
       <c r="BA3" t="n">
-        <v>601.8445400000001</v>
+        <v>640.675219</v>
       </c>
       <c r="BB3" t="n">
-        <v>1.38813184</v>
+        <v>1.26981528</v>
       </c>
       <c r="BC3" t="n">
-        <v>0.0141374667</v>
+        <v>0.0129324684</v>
       </c>
       <c r="BD3" t="n">
-        <v>1.35828246</v>
+        <v>4.40854338</v>
       </c>
       <c r="BE3" t="n">
         <v>15</v>
       </c>
       <c r="BF3" t="n">
-        <v>1.38813184</v>
+        <v>1.26981528</v>
       </c>
       <c r="BG3" t="n">
-        <v>0.0141374667</v>
+        <v>0.0129324684</v>
       </c>
       <c r="BH3" t="n">
-        <v>1.35828246</v>
+        <v>4.40854338</v>
       </c>
       <c r="BI3" t="n">
-        <v>221.706026</v>
+        <v>258.363221</v>
       </c>
       <c r="BJ3" t="n">
-        <v>1.38813184</v>
+        <v>1.26981528</v>
       </c>
       <c r="BK3" t="n">
-        <v>0.0563743756</v>
+        <v>0.0424051433</v>
       </c>
       <c r="BL3" t="n">
-        <v>1.35828246</v>
+        <v>4.40854338</v>
       </c>
       <c r="BM3" t="n">
-        <v>367.905336</v>
+        <v>383.203258</v>
       </c>
       <c r="BN3" t="n">
-        <v>0.00103765376</v>
+        <v>0.0732987378</v>
       </c>
       <c r="BO3" t="n">
-        <v>0.74922176</v>
+        <v>0.695025947</v>
       </c>
       <c r="BP3" t="n">
-        <v>1.38813184</v>
+        <v>1.26981528</v>
       </c>
       <c r="BQ3" t="n">
-        <v>0.0563743756</v>
+        <v>0.0424051433</v>
       </c>
       <c r="BR3" t="n">
-        <v>1.35828246</v>
+        <v>4.40854338</v>
       </c>
       <c r="BS3" t="n">
-        <v>601.658499</v>
+        <v>639.795746</v>
       </c>
       <c r="BT3" t="n">
         <v>70</v>
@@ -1317,7 +1317,7 @@
         <v>50.07</v>
       </c>
       <c r="BW3" t="n">
-        <v>172.813034</v>
+        <v>178.440499</v>
       </c>
       <c r="BX3" t="n">
         <v>70</v>
@@ -1329,7 +1329,7 @@
         <v>50.05</v>
       </c>
       <c r="CA3" t="n">
-        <v>191.585097</v>
+        <v>195.069751</v>
       </c>
       <c r="CB3" t="n">
         <v>70</v>
@@ -1344,27 +1344,27 @@
         <v>264.0032</v>
       </c>
       <c r="CF3" t="n">
-        <v>8.82</v>
+        <v>11.91</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>28</v>
+        <v>66</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8779604059322058</v>
+        <v>0.8170653113087459</v>
       </c>
       <c r="C4" t="n">
-        <v>3.921448287698778</v>
+        <v>4.606822249045958</v>
       </c>
       <c r="D4" t="n">
-        <v>9.395156082207595</v>
+        <v>8.380159647420442</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>7470.98262</v>
+        <v>6302.91111</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -1373,64 +1373,64 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="J4" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="K4" t="n">
-        <v>19.49</v>
+        <v>15</v>
       </c>
       <c r="L4" t="n">
         <v>1500</v>
       </c>
       <c r="M4" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="N4" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="O4" t="n">
         <v>1.034</v>
       </c>
       <c r="P4" t="n">
-        <v>642.22253</v>
+        <v>701.938526</v>
       </c>
       <c r="Q4" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="R4" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="S4" t="n">
         <v>1.027</v>
       </c>
       <c r="T4" t="n">
-        <v>361.02007</v>
+        <v>417.885763</v>
       </c>
       <c r="U4" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="V4" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="W4" t="n">
         <v>1.02</v>
       </c>
       <c r="X4" t="n">
-        <v>204.969845</v>
+        <v>202.913042</v>
       </c>
       <c r="Y4" t="n">
-        <v>313.574709</v>
+        <v>281.840604</v>
       </c>
       <c r="Z4" t="n">
-        <v>11.118118</v>
+        <v>10.0009156</v>
       </c>
       <c r="AA4" t="n">
         <v>1.034</v>
       </c>
       <c r="AB4" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AC4" t="n">
         <v>70</v>
@@ -1442,124 +1442,124 @@
         <v>50</v>
       </c>
       <c r="AF4" t="n">
-        <v>435.134312</v>
+        <v>563.036021</v>
       </c>
       <c r="AG4" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AH4" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AI4" t="n">
         <v>1.013</v>
       </c>
       <c r="AJ4" t="n">
-        <v>190.024085</v>
+        <v>188.351499</v>
       </c>
       <c r="AK4" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AL4" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AM4" t="n">
         <v>1.034</v>
       </c>
       <c r="AN4" t="n">
-        <v>624.96422</v>
+        <v>687.0896</v>
       </c>
       <c r="AO4" t="n">
-        <v>-258041.636</v>
+        <v>-241187.022</v>
       </c>
       <c r="AP4" t="n">
-        <v>-44915.9403</v>
+        <v>-53182.7731</v>
       </c>
       <c r="AQ4" t="n">
-        <v>32.9836374</v>
+        <v>33.7663958</v>
       </c>
       <c r="AR4" t="n">
-        <v>397.141936</v>
+        <v>396.932345</v>
       </c>
       <c r="AS4" t="n">
-        <v>-302527.45</v>
+        <v>-293939.096</v>
       </c>
       <c r="AT4" t="n">
-        <v>43.5879909</v>
+        <v>63.1019607</v>
       </c>
       <c r="AU4" t="n">
-        <v>1.54545764</v>
+        <v>2.2391287</v>
       </c>
       <c r="AV4" t="n">
         <v>1.034</v>
       </c>
       <c r="AW4" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AX4" t="n">
-        <v>43.5879909</v>
+        <v>63.1019607</v>
       </c>
       <c r="AY4" t="n">
-        <v>1.54545764</v>
+        <v>2.2391287</v>
       </c>
       <c r="AZ4" t="n">
         <v>1.034</v>
       </c>
       <c r="BA4" t="n">
-        <v>498.798064</v>
+        <v>620.202312</v>
       </c>
       <c r="BB4" t="n">
-        <v>2.36753951</v>
+        <v>2.11176471</v>
       </c>
       <c r="BC4" t="n">
-        <v>0.0241122708</v>
+        <v>0.0215073254</v>
       </c>
       <c r="BD4" t="n">
-        <v>3.92144829</v>
+        <v>4.60682225</v>
       </c>
       <c r="BE4" t="n">
         <v>15</v>
       </c>
       <c r="BF4" t="n">
-        <v>2.36753951</v>
+        <v>2.11176471</v>
       </c>
       <c r="BG4" t="n">
-        <v>0.0241122708</v>
+        <v>0.0215073254</v>
       </c>
       <c r="BH4" t="n">
-        <v>3.92144829</v>
+        <v>4.60682225</v>
       </c>
       <c r="BI4" t="n">
-        <v>157.344667</v>
+        <v>165.413866</v>
       </c>
       <c r="BJ4" t="n">
-        <v>2.36753951</v>
+        <v>2.11176471</v>
       </c>
       <c r="BK4" t="n">
-        <v>0.09094929810000001</v>
+        <v>0.06931191890000001</v>
       </c>
       <c r="BL4" t="n">
-        <v>3.92144829</v>
+        <v>4.60682225</v>
       </c>
       <c r="BM4" t="n">
-        <v>364.047838</v>
+        <v>440.420552</v>
       </c>
       <c r="BN4" t="n">
-        <v>0.0201569642</v>
+        <v>0.0803968638</v>
       </c>
       <c r="BO4" t="n">
-        <v>0.734882277</v>
+        <v>0.689702352</v>
       </c>
       <c r="BP4" t="n">
-        <v>2.36753951</v>
+        <v>2.11176471</v>
       </c>
       <c r="BQ4" t="n">
-        <v>0.09094929810000001</v>
+        <v>0.06931191890000001</v>
       </c>
       <c r="BR4" t="n">
-        <v>3.92144829</v>
+        <v>4.60682225</v>
       </c>
       <c r="BS4" t="n">
-        <v>496.842763</v>
+        <v>619.050734</v>
       </c>
       <c r="BT4" t="n">
         <v>70</v>
@@ -1571,7 +1571,7 @@
         <v>50.07</v>
       </c>
       <c r="BW4" t="n">
-        <v>172.035093</v>
+        <v>171.577382</v>
       </c>
       <c r="BX4" t="n">
         <v>70</v>
@@ -1583,7 +1583,7 @@
         <v>50.05</v>
       </c>
       <c r="CA4" t="n">
-        <v>191.016204</v>
+        <v>189.554622</v>
       </c>
       <c r="CB4" t="n">
         <v>70</v>
@@ -1598,27 +1598,27 @@
         <v>264.0032</v>
       </c>
       <c r="CF4" t="n">
-        <v>12.76</v>
+        <v>12.31</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B5" t="n">
-        <v>0.7210266119912327</v>
+        <v>0.8067830825533916</v>
       </c>
       <c r="C5" t="n">
-        <v>4.946846213273429</v>
+        <v>1.412343773778501</v>
       </c>
       <c r="D5" t="n">
-        <v>14.21559273672534</v>
+        <v>12.18423151176027</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>11037.0777</v>
+        <v>10867.0535</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -1627,64 +1627,64 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="J5" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="K5" t="n">
-        <v>19.49</v>
+        <v>15</v>
       </c>
       <c r="L5" t="n">
         <v>1500</v>
       </c>
       <c r="M5" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="N5" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="O5" t="n">
         <v>1.034</v>
       </c>
       <c r="P5" t="n">
-        <v>642.22253</v>
+        <v>701.938526</v>
       </c>
       <c r="Q5" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="R5" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="S5" t="n">
         <v>1.027</v>
       </c>
       <c r="T5" t="n">
-        <v>352.718281</v>
+        <v>403.038296</v>
       </c>
       <c r="U5" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="V5" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="W5" t="n">
         <v>1.02</v>
       </c>
       <c r="X5" t="n">
-        <v>204.520321</v>
+        <v>205.907273</v>
       </c>
       <c r="Y5" t="n">
-        <v>257.523811</v>
+        <v>278.293826</v>
       </c>
       <c r="Z5" t="n">
-        <v>9.13077507</v>
+        <v>9.875060700000001</v>
       </c>
       <c r="AA5" t="n">
         <v>1.034</v>
       </c>
       <c r="AB5" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AC5" t="n">
         <v>70</v>
@@ -1696,124 +1696,124 @@
         <v>50</v>
       </c>
       <c r="AF5" t="n">
-        <v>413.81182</v>
+        <v>535.124215</v>
       </c>
       <c r="AG5" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AH5" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AI5" t="n">
         <v>1.013</v>
       </c>
       <c r="AJ5" t="n">
-        <v>189.337658</v>
+        <v>192.222508</v>
       </c>
       <c r="AK5" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AL5" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AM5" t="n">
         <v>1.034</v>
       </c>
       <c r="AN5" t="n">
-        <v>616.703581</v>
+        <v>676.308885</v>
       </c>
       <c r="AO5" t="n">
-        <v>-258041.636</v>
+        <v>-241187.022</v>
       </c>
       <c r="AP5" t="n">
-        <v>-43646.8855</v>
+        <v>-50888.2094</v>
       </c>
       <c r="AQ5" t="n">
         <v>32.9836374</v>
       </c>
       <c r="AR5" t="n">
-        <v>396.695561</v>
+        <v>399.22222</v>
       </c>
       <c r="AS5" t="n">
-        <v>-301258.842</v>
+        <v>-291643.025</v>
       </c>
       <c r="AT5" t="n">
-        <v>99.6388884</v>
+        <v>66.64873900000001</v>
       </c>
       <c r="AU5" t="n">
-        <v>3.53280061</v>
+        <v>2.36498363</v>
       </c>
       <c r="AV5" t="n">
         <v>1.034</v>
       </c>
       <c r="AW5" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AX5" t="n">
-        <v>99.6388884</v>
+        <v>66.64873900000001</v>
       </c>
       <c r="AY5" t="n">
-        <v>3.53280061</v>
+        <v>2.36498363</v>
       </c>
       <c r="AZ5" t="n">
         <v>1.034</v>
       </c>
       <c r="BA5" t="n">
-        <v>550.071918</v>
+        <v>567.7568240000001</v>
       </c>
       <c r="BB5" t="n">
-        <v>3.58226911</v>
+        <v>3.07037469</v>
       </c>
       <c r="BC5" t="n">
-        <v>0.0364837177</v>
+        <v>0.031270315</v>
       </c>
       <c r="BD5" t="n">
-        <v>4.94684621</v>
+        <v>1.41234377</v>
       </c>
       <c r="BE5" t="n">
         <v>15</v>
       </c>
       <c r="BF5" t="n">
-        <v>3.58226911</v>
+        <v>3.07037469</v>
       </c>
       <c r="BG5" t="n">
-        <v>0.0364837177</v>
+        <v>0.031270315</v>
       </c>
       <c r="BH5" t="n">
-        <v>4.94684621</v>
+        <v>1.41234377</v>
       </c>
       <c r="BI5" t="n">
-        <v>155.747445</v>
+        <v>112.987131</v>
       </c>
       <c r="BJ5" t="n">
-        <v>3.58226911</v>
+        <v>3.07037469</v>
       </c>
       <c r="BK5" t="n">
-        <v>0.12130728</v>
+        <v>0.124196285</v>
       </c>
       <c r="BL5" t="n">
-        <v>4.94684621</v>
+        <v>1.41234377</v>
       </c>
       <c r="BM5" t="n">
-        <v>447.229863</v>
+        <v>441.757197</v>
       </c>
       <c r="BN5" t="n">
-        <v>0.06767274719999999</v>
+        <v>0.00237520403</v>
       </c>
       <c r="BO5" t="n">
-        <v>0.69924544</v>
+        <v>0.748218597</v>
       </c>
       <c r="BP5" t="n">
-        <v>3.58226911</v>
+        <v>3.07037469</v>
       </c>
       <c r="BQ5" t="n">
-        <v>0.12130728</v>
+        <v>0.124196285</v>
       </c>
       <c r="BR5" t="n">
-        <v>4.94684621</v>
+        <v>1.41234377</v>
       </c>
       <c r="BS5" t="n">
-        <v>547.90019</v>
+        <v>567.154882</v>
       </c>
       <c r="BT5" t="n">
         <v>70</v>
@@ -1825,7 +1825,7 @@
         <v>50.07</v>
       </c>
       <c r="BW5" t="n">
-        <v>171.058521</v>
+        <v>176.50022</v>
       </c>
       <c r="BX5" t="n">
         <v>70</v>
@@ -1837,7 +1837,7 @@
         <v>50.05</v>
       </c>
       <c r="CA5" t="n">
-        <v>190.352764</v>
+        <v>193.316475</v>
       </c>
       <c r="CB5" t="n">
         <v>70</v>
@@ -1852,27 +1852,27 @@
         <v>264.0032</v>
       </c>
       <c r="CF5" t="n">
-        <v>10.44</v>
+        <v>11.77</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="B6" t="n">
-        <v>0.8862135875635846</v>
+        <v>0.9458997340379108</v>
       </c>
       <c r="C6" t="n">
-        <v>3.587417758128223</v>
+        <v>2.568131955354081</v>
       </c>
       <c r="D6" t="n">
-        <v>18.20474868637531</v>
+        <v>15.26368854762517</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>13899.3261</v>
+        <v>8892.455959999999</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -1881,64 +1881,64 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="J6" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="K6" t="n">
-        <v>19.49</v>
+        <v>15</v>
       </c>
       <c r="L6" t="n">
         <v>1500</v>
       </c>
       <c r="M6" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="N6" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="O6" t="n">
         <v>1.034</v>
       </c>
       <c r="P6" t="n">
-        <v>642.22253</v>
+        <v>701.938526</v>
       </c>
       <c r="Q6" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="R6" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="S6" t="n">
         <v>1.027</v>
       </c>
       <c r="T6" t="n">
-        <v>346.44525</v>
+        <v>409.260878</v>
       </c>
       <c r="U6" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="V6" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="W6" t="n">
         <v>1.02</v>
       </c>
       <c r="X6" t="n">
-        <v>204.228164</v>
+        <v>206.391313</v>
       </c>
       <c r="Y6" t="n">
-        <v>316.522437</v>
+        <v>326.28108</v>
       </c>
       <c r="Z6" t="n">
-        <v>11.2226328</v>
+        <v>11.5778547</v>
       </c>
       <c r="AA6" t="n">
         <v>1.034</v>
       </c>
       <c r="AB6" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AC6" t="n">
         <v>70</v>
@@ -1950,124 +1950,124 @@
         <v>50</v>
       </c>
       <c r="AF6" t="n">
-        <v>396.879366</v>
+        <v>547.106655</v>
       </c>
       <c r="AG6" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AH6" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AI6" t="n">
         <v>1.013</v>
       </c>
       <c r="AJ6" t="n">
-        <v>188.822201</v>
+        <v>192.730797</v>
       </c>
       <c r="AK6" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AL6" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AM6" t="n">
         <v>1.034</v>
       </c>
       <c r="AN6" t="n">
-        <v>610.062552</v>
+        <v>680.975906</v>
       </c>
       <c r="AO6" t="n">
-        <v>-258041.636</v>
+        <v>-241187.022</v>
       </c>
       <c r="AP6" t="n">
-        <v>-42635.0291</v>
+        <v>-51612.4461</v>
       </c>
       <c r="AQ6" t="n">
         <v>32.9836374</v>
       </c>
       <c r="AR6" t="n">
-        <v>396.337498</v>
+        <v>399.4737</v>
       </c>
       <c r="AS6" t="n">
-        <v>-300247.344</v>
+        <v>-292367.01</v>
       </c>
       <c r="AT6" t="n">
-        <v>40.6402623</v>
+        <v>18.6614845</v>
       </c>
       <c r="AU6" t="n">
-        <v>1.44094285</v>
+        <v>0.662189654</v>
       </c>
       <c r="AV6" t="n">
         <v>1.034</v>
       </c>
       <c r="AW6" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AX6" t="n">
-        <v>40.6402623</v>
+        <v>18.6614845</v>
       </c>
       <c r="AY6" t="n">
-        <v>1.44094285</v>
+        <v>0.662189654</v>
       </c>
       <c r="AZ6" t="n">
         <v>1.034</v>
       </c>
       <c r="BA6" t="n">
-        <v>350.988222</v>
+        <v>297.308651</v>
       </c>
       <c r="BB6" t="n">
-        <v>4.5875195</v>
+        <v>3.84638481</v>
       </c>
       <c r="BC6" t="n">
-        <v>0.0467217178</v>
+        <v>0.0391736113</v>
       </c>
       <c r="BD6" t="n">
-        <v>3.58741776</v>
+        <v>2.56813196</v>
       </c>
       <c r="BE6" t="n">
         <v>15</v>
       </c>
       <c r="BF6" t="n">
-        <v>4.5875195</v>
+        <v>3.84638481</v>
       </c>
       <c r="BG6" t="n">
-        <v>0.0467217178</v>
+        <v>0.0391736113</v>
       </c>
       <c r="BH6" t="n">
-        <v>3.58741776</v>
+        <v>2.56813196</v>
       </c>
       <c r="BI6" t="n">
-        <v>92.3066001</v>
+        <v>89.8290216</v>
       </c>
       <c r="BJ6" t="n">
-        <v>4.5875195</v>
+        <v>3.84638481</v>
       </c>
       <c r="BK6" t="n">
-        <v>0.181631153</v>
+        <v>0.121378917</v>
       </c>
       <c r="BL6" t="n">
-        <v>3.58741776</v>
+        <v>2.56813196</v>
       </c>
       <c r="BM6" t="n">
-        <v>291.026479</v>
+        <v>237.840478</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.009645405120000001</v>
+        <v>0.09698424429999999</v>
       </c>
       <c r="BO6" t="n">
-        <v>0.742765946</v>
+        <v>0.677261817</v>
       </c>
       <c r="BP6" t="n">
-        <v>4.5875195</v>
+        <v>3.84638481</v>
       </c>
       <c r="BQ6" t="n">
-        <v>0.181631153</v>
+        <v>0.121378917</v>
       </c>
       <c r="BR6" t="n">
-        <v>3.58741776</v>
+        <v>2.56813196</v>
       </c>
       <c r="BS6" t="n">
-        <v>348.508538</v>
+        <v>297.202859</v>
       </c>
       <c r="BT6" t="n">
         <v>70</v>
@@ -2079,7 +2079,7 @@
         <v>50.07</v>
       </c>
       <c r="BW6" t="n">
-        <v>170.270321</v>
+        <v>177.030613</v>
       </c>
       <c r="BX6" t="n">
         <v>70</v>
@@ -2091,7 +2091,7 @@
         <v>50.05</v>
       </c>
       <c r="CA6" t="n">
-        <v>189.857859</v>
+        <v>193.818948</v>
       </c>
       <c r="CB6" t="n">
         <v>70</v>
@@ -2106,27 +2106,27 @@
         <v>264.0032</v>
       </c>
       <c r="CF6" t="n">
-        <v>12.07</v>
+        <v>11.45</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="B7" t="n">
-        <v>0.9152050879042952</v>
+        <v>0.7147138793840611</v>
       </c>
       <c r="C7" t="n">
-        <v>4.506722750882067</v>
+        <v>1.395261646125348</v>
       </c>
       <c r="D7" t="n">
-        <v>22.20759575533632</v>
+        <v>19.11058620244465</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>11738.386</v>
+        <v>17490.4804</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -2135,64 +2135,64 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="J7" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="K7" t="n">
-        <v>19.49</v>
+        <v>15</v>
       </c>
       <c r="L7" t="n">
         <v>1500</v>
       </c>
       <c r="M7" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="N7" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="O7" t="n">
         <v>1.034</v>
       </c>
       <c r="P7" t="n">
-        <v>642.22253</v>
+        <v>701.938526</v>
       </c>
       <c r="Q7" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="R7" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="S7" t="n">
         <v>1.027</v>
       </c>
       <c r="T7" t="n">
-        <v>351.14959</v>
+        <v>383.584068</v>
       </c>
       <c r="U7" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="V7" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="W7" t="n">
         <v>1.02</v>
       </c>
       <c r="X7" t="n">
-        <v>204.443081</v>
+        <v>204.468191</v>
       </c>
       <c r="Y7" t="n">
-        <v>326.87712</v>
+        <v>246.535238</v>
       </c>
       <c r="Z7" t="n">
-        <v>11.5897689</v>
+        <v>8.74812957</v>
       </c>
       <c r="AA7" t="n">
         <v>1.034</v>
       </c>
       <c r="AB7" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AC7" t="n">
         <v>70</v>
@@ -2204,124 +2204,124 @@
         <v>50</v>
       </c>
       <c r="AF7" t="n">
-        <v>409.645787</v>
+        <v>494.773001</v>
       </c>
       <c r="AG7" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AH7" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AI7" t="n">
         <v>1.013</v>
       </c>
       <c r="AJ7" t="n">
-        <v>189.208458</v>
+        <v>190.607479</v>
       </c>
       <c r="AK7" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AL7" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AM7" t="n">
         <v>1.034</v>
       </c>
       <c r="AN7" t="n">
-        <v>615.0772899999999</v>
+        <v>660.6211479999999</v>
       </c>
       <c r="AO7" t="n">
-        <v>-258041.636</v>
+        <v>-241187.022</v>
       </c>
       <c r="AP7" t="n">
-        <v>-43398.3857</v>
+        <v>-48466.0071</v>
       </c>
       <c r="AQ7" t="n">
         <v>32.9836374</v>
       </c>
       <c r="AR7" t="n">
-        <v>396.607824</v>
+        <v>398.380766</v>
       </c>
       <c r="AS7" t="n">
-        <v>-301010.43</v>
+        <v>-289221.664</v>
       </c>
       <c r="AT7" t="n">
-        <v>30.2855797</v>
+        <v>98.40732610000001</v>
       </c>
       <c r="AU7" t="n">
-        <v>1.07380679</v>
+        <v>3.49191476</v>
       </c>
       <c r="AV7" t="n">
         <v>1.034</v>
       </c>
       <c r="AW7" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AX7" t="n">
-        <v>30.2855797</v>
+        <v>98.40732610000001</v>
       </c>
       <c r="AY7" t="n">
-        <v>1.07380679</v>
+        <v>3.49191476</v>
       </c>
       <c r="AZ7" t="n">
         <v>1.034</v>
       </c>
       <c r="BA7" t="n">
-        <v>310.568353</v>
+        <v>555.473355</v>
       </c>
       <c r="BB7" t="n">
-        <v>5.59621999</v>
+        <v>4.81578672</v>
       </c>
       <c r="BC7" t="n">
-        <v>0.0569948555</v>
+        <v>0.0490465115</v>
       </c>
       <c r="BD7" t="n">
-        <v>4.50672275</v>
+        <v>1.39526165</v>
       </c>
       <c r="BE7" t="n">
         <v>15</v>
       </c>
       <c r="BF7" t="n">
-        <v>5.59621999</v>
+        <v>4.81578672</v>
       </c>
       <c r="BG7" t="n">
-        <v>0.0569948555</v>
+        <v>0.0490465115</v>
       </c>
       <c r="BH7" t="n">
-        <v>4.50672275</v>
+        <v>1.39526165</v>
       </c>
       <c r="BI7" t="n">
-        <v>74.03896810000001</v>
+        <v>112.521129</v>
       </c>
       <c r="BJ7" t="n">
-        <v>5.59621999</v>
+        <v>4.81578672</v>
       </c>
       <c r="BK7" t="n">
-        <v>0.15454799</v>
+        <v>0.194365709</v>
       </c>
       <c r="BL7" t="n">
-        <v>4.50672275</v>
+        <v>1.39526165</v>
       </c>
       <c r="BM7" t="n">
-        <v>263.526431</v>
+        <v>473.125355</v>
       </c>
       <c r="BN7" t="n">
-        <v>0.158378922</v>
+        <v>0.00312184161</v>
       </c>
       <c r="BO7" t="n">
-        <v>0.631215808</v>
+        <v>0.747658619</v>
       </c>
       <c r="BP7" t="n">
-        <v>5.59621999</v>
+        <v>4.81578672</v>
       </c>
       <c r="BQ7" t="n">
-        <v>0.15454799</v>
+        <v>0.194365709</v>
       </c>
       <c r="BR7" t="n">
-        <v>4.50672275</v>
+        <v>1.39526165</v>
       </c>
       <c r="BS7" t="n">
-        <v>308.869989</v>
+        <v>554.411526</v>
       </c>
       <c r="BT7" t="n">
         <v>70</v>
@@ -2333,7 +2333,7 @@
         <v>50.07</v>
       </c>
       <c r="BW7" t="n">
-        <v>170.865787</v>
+        <v>174.710955</v>
       </c>
       <c r="BX7" t="n">
         <v>70</v>
@@ -2345,7 +2345,7 @@
         <v>50.05</v>
       </c>
       <c r="CA7" t="n">
-        <v>190.228423</v>
+        <v>191.727417</v>
       </c>
       <c r="CB7" t="n">
         <v>70</v>
@@ -2360,27 +2360,27 @@
         <v>264.0032</v>
       </c>
       <c r="CF7" t="n">
-        <v>11.67</v>
+        <v>10.86</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="B8" t="n">
-        <v>0.8589235585477533</v>
+        <v>0.9152050879042952</v>
       </c>
       <c r="C8" t="n">
-        <v>3.894933630563157</v>
+        <v>4.506722750882067</v>
       </c>
       <c r="D8" t="n">
-        <v>26.58724443486842</v>
+        <v>22.20759575533632</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>18026.3958</v>
+        <v>13210.6457</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -2389,64 +2389,64 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="J8" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="K8" t="n">
-        <v>19.49</v>
+        <v>15</v>
       </c>
       <c r="L8" t="n">
         <v>1500</v>
       </c>
       <c r="M8" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="N8" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="O8" t="n">
         <v>1.034</v>
       </c>
       <c r="P8" t="n">
-        <v>642.22253</v>
+        <v>701.938526</v>
       </c>
       <c r="Q8" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="R8" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="S8" t="n">
         <v>1.027</v>
       </c>
       <c r="T8" t="n">
-        <v>337.973438</v>
+        <v>395.911023</v>
       </c>
       <c r="U8" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="V8" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="W8" t="n">
         <v>1.02</v>
       </c>
       <c r="X8" t="n">
-        <v>200.751502</v>
+        <v>205.367535</v>
       </c>
       <c r="Y8" t="n">
-        <v>306.775457</v>
+        <v>315.69319</v>
       </c>
       <c r="Z8" t="n">
-        <v>10.8770435</v>
+        <v>11.2021508</v>
       </c>
       <c r="AA8" t="n">
         <v>1.034</v>
       </c>
       <c r="AB8" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AC8" t="n">
         <v>70</v>
@@ -2458,124 +2458,124 @@
         <v>50</v>
       </c>
       <c r="AF8" t="n">
-        <v>372.750835</v>
+        <v>520.868006</v>
       </c>
       <c r="AG8" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AH8" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AI8" t="n">
         <v>1.013</v>
       </c>
       <c r="AJ8" t="n">
-        <v>183.920242</v>
+        <v>191.637611</v>
       </c>
       <c r="AK8" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AL8" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AM8" t="n">
         <v>1.034</v>
       </c>
       <c r="AN8" t="n">
-        <v>600.469732</v>
+        <v>670.763887</v>
       </c>
       <c r="AO8" t="n">
-        <v>-258041.636</v>
+        <v>-241187.022</v>
       </c>
       <c r="AP8" t="n">
-        <v>-41689.6717</v>
+        <v>-50029.6922</v>
       </c>
       <c r="AQ8" t="n">
-        <v>33.7663958</v>
+        <v>32.9836374</v>
       </c>
       <c r="AR8" t="n">
-        <v>393.394418</v>
+        <v>398.924097</v>
       </c>
       <c r="AS8" t="n">
-        <v>-299304.146</v>
+        <v>-290784.806</v>
       </c>
       <c r="AT8" t="n">
-        <v>50.3872427</v>
+        <v>29.2493744</v>
       </c>
       <c r="AU8" t="n">
-        <v>1.78653219</v>
+        <v>1.03789348</v>
       </c>
       <c r="AV8" t="n">
         <v>1.034</v>
       </c>
       <c r="AW8" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AX8" t="n">
-        <v>50.3872427</v>
+        <v>29.2493744</v>
       </c>
       <c r="AY8" t="n">
-        <v>1.78653219</v>
+        <v>1.03789348</v>
       </c>
       <c r="AZ8" t="n">
         <v>1.034</v>
       </c>
       <c r="BA8" t="n">
-        <v>337.068186</v>
+        <v>319.424349</v>
       </c>
       <c r="BB8" t="n">
-        <v>6.6998729</v>
+        <v>5.59621999</v>
       </c>
       <c r="BC8" t="n">
-        <v>0.0682350387</v>
+        <v>0.0569948555</v>
       </c>
       <c r="BD8" t="n">
-        <v>3.89493363</v>
+        <v>4.50672275</v>
       </c>
       <c r="BE8" t="n">
         <v>15</v>
       </c>
       <c r="BF8" t="n">
-        <v>6.6998729</v>
+        <v>5.59621999</v>
       </c>
       <c r="BG8" t="n">
-        <v>0.0682350387</v>
+        <v>0.0569948555</v>
       </c>
       <c r="BH8" t="n">
-        <v>3.89493363</v>
+        <v>4.50672275</v>
       </c>
       <c r="BI8" t="n">
-        <v>69.01982169999999</v>
+        <v>75.7384945</v>
       </c>
       <c r="BJ8" t="n">
-        <v>6.6998729</v>
+        <v>5.59621999</v>
       </c>
       <c r="BK8" t="n">
-        <v>0.235084248</v>
+        <v>0.173447812</v>
       </c>
       <c r="BL8" t="n">
-        <v>3.89493363</v>
+        <v>4.50672275</v>
       </c>
       <c r="BM8" t="n">
-        <v>285.088171</v>
+        <v>271.59094</v>
       </c>
       <c r="BN8" t="n">
-        <v>0.0536770779</v>
+        <v>0.104799265</v>
       </c>
       <c r="BO8" t="n">
-        <v>0.709742192</v>
+        <v>0.671400551</v>
       </c>
       <c r="BP8" t="n">
-        <v>6.6998729</v>
+        <v>5.59621999</v>
       </c>
       <c r="BQ8" t="n">
-        <v>0.235084248</v>
+        <v>0.173447812</v>
       </c>
       <c r="BR8" t="n">
-        <v>3.89493363</v>
+        <v>4.50672275</v>
       </c>
       <c r="BS8" t="n">
-        <v>324.85916</v>
+        <v>317.569346</v>
       </c>
       <c r="BT8" t="n">
         <v>70</v>
@@ -2587,7 +2587,7 @@
         <v>50.07</v>
       </c>
       <c r="BW8" t="n">
-        <v>163.623147</v>
+        <v>175.868869</v>
       </c>
       <c r="BX8" t="n">
         <v>70</v>
@@ -2599,7 +2599,7 @@
         <v>50.05</v>
       </c>
       <c r="CA8" t="n">
-        <v>185.105546</v>
+        <v>192.739716</v>
       </c>
       <c r="CB8" t="n">
         <v>70</v>
@@ -2614,27 +2614,27 @@
         <v>264.0032</v>
       </c>
       <c r="CF8" t="n">
-        <v>9.51</v>
+        <v>11.44</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="B9" t="n">
-        <v>0.8463446545163971</v>
+        <v>0.7890420854183274</v>
       </c>
       <c r="C9" t="n">
-        <v>4.06503856930946</v>
+        <v>3.073092187666094</v>
       </c>
       <c r="D9" t="n">
-        <v>33.44694037783154</v>
+        <v>25.57829564080328</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>19978.3811</v>
+        <v>21458.4231</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -2643,64 +2643,64 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="J9" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="K9" t="n">
-        <v>19.49</v>
+        <v>15</v>
       </c>
       <c r="L9" t="n">
         <v>1500</v>
       </c>
       <c r="M9" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="N9" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="O9" t="n">
         <v>1.034</v>
       </c>
       <c r="P9" t="n">
-        <v>642.22253</v>
+        <v>701.938526</v>
       </c>
       <c r="Q9" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="R9" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="S9" t="n">
         <v>1.027</v>
       </c>
       <c r="T9" t="n">
-        <v>334.229914</v>
+        <v>372.923184</v>
       </c>
       <c r="U9" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="V9" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="W9" t="n">
         <v>1.02</v>
       </c>
       <c r="X9" t="n">
-        <v>200.706098</v>
+        <v>203.764397</v>
       </c>
       <c r="Y9" t="n">
-        <v>302.282742</v>
+        <v>272.1742</v>
       </c>
       <c r="Z9" t="n">
-        <v>10.7177496</v>
+        <v>9.6579101</v>
       </c>
       <c r="AA9" t="n">
         <v>1.034</v>
       </c>
       <c r="AB9" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AC9" t="n">
         <v>70</v>
@@ -2712,124 +2712,124 @@
         <v>50</v>
       </c>
       <c r="AF9" t="n">
-        <v>361.611361</v>
+        <v>470.597657</v>
       </c>
       <c r="AG9" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AH9" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AI9" t="n">
         <v>1.013</v>
       </c>
       <c r="AJ9" t="n">
-        <v>183.667987</v>
+        <v>189.730151</v>
       </c>
       <c r="AK9" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AL9" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AM9" t="n">
         <v>1.034</v>
       </c>
       <c r="AN9" t="n">
-        <v>595.925486</v>
+        <v>651.198299</v>
       </c>
       <c r="AO9" t="n">
-        <v>-258041.636</v>
+        <v>-241187.022</v>
       </c>
       <c r="AP9" t="n">
-        <v>-41005.2982</v>
+        <v>-47024.4411</v>
       </c>
       <c r="AQ9" t="n">
-        <v>33.7663958</v>
+        <v>32.9836374</v>
       </c>
       <c r="AR9" t="n">
-        <v>393.176826</v>
+        <v>397.878956</v>
       </c>
       <c r="AS9" t="n">
-        <v>-298619.991</v>
+        <v>-287780.6</v>
       </c>
       <c r="AT9" t="n">
-        <v>54.879958</v>
+        <v>72.7683641</v>
       </c>
       <c r="AU9" t="n">
-        <v>1.9458261</v>
+        <v>2.58213423</v>
       </c>
       <c r="AV9" t="n">
         <v>1.034</v>
       </c>
       <c r="AW9" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AX9" t="n">
-        <v>54.879958</v>
+        <v>72.7683641</v>
       </c>
       <c r="AY9" t="n">
-        <v>1.9458261</v>
+        <v>2.58213423</v>
       </c>
       <c r="AZ9" t="n">
         <v>1.034</v>
       </c>
       <c r="BA9" t="n">
-        <v>331.503374</v>
+        <v>456.187696</v>
       </c>
       <c r="BB9" t="n">
-        <v>8.428487199999999</v>
+        <v>6.44562208</v>
       </c>
       <c r="BC9" t="n">
-        <v>0.0858401583</v>
+        <v>0.0656456143</v>
       </c>
       <c r="BD9" t="n">
-        <v>4.06503857</v>
+        <v>3.07309219</v>
       </c>
       <c r="BE9" t="n">
         <v>15</v>
       </c>
       <c r="BF9" t="n">
-        <v>8.428487199999999</v>
+        <v>6.44562208</v>
       </c>
       <c r="BG9" t="n">
-        <v>0.0858401583</v>
+        <v>0.0656456143</v>
       </c>
       <c r="BH9" t="n">
-        <v>4.06503857</v>
+        <v>3.07309219</v>
       </c>
       <c r="BI9" t="n">
-        <v>58.2666383</v>
+        <v>91.8885677</v>
       </c>
       <c r="BJ9" t="n">
-        <v>8.428487199999999</v>
+        <v>6.44562208</v>
       </c>
       <c r="BK9" t="n">
-        <v>0.259119262</v>
+        <v>0.253868684</v>
       </c>
       <c r="BL9" t="n">
-        <v>4.06503857</v>
+        <v>3.07309219</v>
       </c>
       <c r="BM9" t="n">
-        <v>281.826105</v>
+        <v>398.57243</v>
       </c>
       <c r="BN9" t="n">
-        <v>0.108368853</v>
+        <v>0.011441313</v>
       </c>
       <c r="BO9" t="n">
-        <v>0.668723361</v>
+        <v>0.741419015</v>
       </c>
       <c r="BP9" t="n">
-        <v>8.428487199999999</v>
+        <v>6.44562208</v>
       </c>
       <c r="BQ9" t="n">
-        <v>0.259119262</v>
+        <v>0.253868684</v>
       </c>
       <c r="BR9" t="n">
-        <v>4.06503857</v>
+        <v>3.07309219</v>
       </c>
       <c r="BS9" t="n">
-        <v>313.731928</v>
+        <v>451.411315</v>
       </c>
       <c r="BT9" t="n">
         <v>70</v>
@@ -2841,7 +2841,7 @@
         <v>50.07</v>
       </c>
       <c r="BW9" t="n">
-        <v>163.119376</v>
+        <v>173.633088</v>
       </c>
       <c r="BX9" t="n">
         <v>70</v>
@@ -2853,7 +2853,7 @@
         <v>50.05</v>
       </c>
       <c r="CA9" t="n">
-        <v>184.871001</v>
+        <v>190.871873</v>
       </c>
       <c r="CB9" t="n">
         <v>70</v>
@@ -2868,27 +2868,27 @@
         <v>264.0032</v>
       </c>
       <c r="CF9" t="n">
-        <v>11.47</v>
+        <v>11.72</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>62</v>
+        <v>17</v>
       </c>
       <c r="B10" t="n">
-        <v>0.977880327309136</v>
+        <v>0.9225985530409572</v>
       </c>
       <c r="C10" t="n">
-        <v>1.233844534766142</v>
+        <v>3.692273252062969</v>
       </c>
       <c r="D10" t="n">
-        <v>40.70086157381182</v>
+        <v>29.32743059811902</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>4821.34075</v>
+        <v>12926.5448</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -2897,64 +2897,64 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="J10" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="K10" t="n">
-        <v>19.49</v>
+        <v>15</v>
       </c>
       <c r="L10" t="n">
         <v>1500</v>
       </c>
       <c r="M10" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="N10" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="O10" t="n">
         <v>1.034</v>
       </c>
       <c r="P10" t="n">
-        <v>642.22253</v>
+        <v>701.938526</v>
       </c>
       <c r="Q10" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="R10" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="S10" t="n">
         <v>1.027</v>
       </c>
       <c r="T10" t="n">
-        <v>367.54755</v>
+        <v>396.760265</v>
       </c>
       <c r="U10" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="V10" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="W10" t="n">
         <v>1.02</v>
       </c>
       <c r="X10" t="n">
-        <v>205.365182</v>
+        <v>205.431001</v>
       </c>
       <c r="Y10" t="n">
-        <v>349.262378</v>
+        <v>318.243511</v>
       </c>
       <c r="Z10" t="n">
-        <v>12.3834615</v>
+        <v>11.2926472</v>
       </c>
       <c r="AA10" t="n">
         <v>1.034</v>
       </c>
       <c r="AB10" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AC10" t="n">
         <v>70</v>
@@ -2966,124 +2966,124 @@
         <v>50</v>
       </c>
       <c r="AF10" t="n">
-        <v>451.087789</v>
+        <v>522.5974629999999</v>
       </c>
       <c r="AG10" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AH10" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AI10" t="n">
         <v>1.013</v>
       </c>
       <c r="AJ10" t="n">
-        <v>190.566176</v>
+        <v>191.707513</v>
       </c>
       <c r="AK10" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AL10" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AM10" t="n">
         <v>1.034</v>
       </c>
       <c r="AN10" t="n">
-        <v>631.0923739999999</v>
+        <v>671.436417</v>
       </c>
       <c r="AO10" t="n">
-        <v>-258041.636</v>
+        <v>-241187.022</v>
       </c>
       <c r="AP10" t="n">
-        <v>-45864.1407</v>
+        <v>-50133.6707</v>
       </c>
       <c r="AQ10" t="n">
         <v>32.9836374</v>
       </c>
       <c r="AR10" t="n">
-        <v>397.473954</v>
+        <v>398.960206</v>
       </c>
       <c r="AS10" t="n">
-        <v>-303475.319</v>
+        <v>-290888.748</v>
       </c>
       <c r="AT10" t="n">
-        <v>7.90032201</v>
+        <v>26.6990536</v>
       </c>
       <c r="AU10" t="n">
-        <v>0.280114149</v>
+        <v>0.947397142</v>
       </c>
       <c r="AV10" t="n">
         <v>1.034</v>
       </c>
       <c r="AW10" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AX10" t="n">
-        <v>7.90032201</v>
+        <v>26.6990536</v>
       </c>
       <c r="AY10" t="n">
-        <v>0.280114149</v>
+        <v>0.947397142</v>
       </c>
       <c r="AZ10" t="n">
         <v>1.034</v>
       </c>
       <c r="BA10" t="n">
-        <v>107.646643</v>
+        <v>290.484691</v>
       </c>
       <c r="BB10" t="n">
-        <v>10.2564446</v>
+        <v>7.39038819</v>
       </c>
       <c r="BC10" t="n">
-        <v>0.10445704</v>
+        <v>0.07526761060000001</v>
       </c>
       <c r="BD10" t="n">
-        <v>1.23384453</v>
+        <v>3.69227325</v>
       </c>
       <c r="BE10" t="n">
         <v>15</v>
       </c>
       <c r="BF10" t="n">
-        <v>10.2564446</v>
+        <v>7.39038819</v>
       </c>
       <c r="BG10" t="n">
-        <v>0.10445704</v>
+        <v>0.07526761060000001</v>
       </c>
       <c r="BH10" t="n">
-        <v>1.23384453</v>
+        <v>3.69227325</v>
       </c>
       <c r="BI10" t="n">
-        <v>27.2437828</v>
+        <v>59.3223472</v>
       </c>
       <c r="BJ10" t="n">
-        <v>10.2564446</v>
+        <v>7.39038819</v>
       </c>
       <c r="BK10" t="n">
-        <v>0.105146607</v>
+        <v>0.170391695</v>
       </c>
       <c r="BL10" t="n">
-        <v>1.23384453</v>
+        <v>3.69227325</v>
       </c>
       <c r="BM10" t="n">
-        <v>107.621791</v>
+        <v>254.907651</v>
       </c>
       <c r="BN10" t="n">
-        <v>0.99125581</v>
+        <v>0.255643813</v>
       </c>
       <c r="BO10" t="n">
-        <v>0.00655814259</v>
+        <v>0.55826714</v>
       </c>
       <c r="BP10" t="n">
-        <v>10.2564446</v>
+        <v>7.39038819</v>
       </c>
       <c r="BQ10" t="n">
-        <v>0.105146607</v>
+        <v>0.170391695</v>
       </c>
       <c r="BR10" t="n">
-        <v>1.23384453</v>
+        <v>3.69227325</v>
       </c>
       <c r="BS10" t="n">
-        <v>107.646214</v>
+        <v>289.246339</v>
       </c>
       <c r="BT10" t="n">
         <v>70</v>
@@ -3095,7 +3095,7 @@
         <v>50.07</v>
       </c>
       <c r="BW10" t="n">
-        <v>172.757182</v>
+        <v>175.945489</v>
       </c>
       <c r="BX10" t="n">
         <v>70</v>
@@ -3107,7 +3107,7 @@
         <v>50.05</v>
       </c>
       <c r="CA10" t="n">
-        <v>191.543073</v>
+        <v>192.808563</v>
       </c>
       <c r="CB10" t="n">
         <v>70</v>
@@ -3122,27 +3122,27 @@
         <v>264.0032</v>
       </c>
       <c r="CF10" t="n">
-        <v>12.09</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>4</v>
+        <v>88</v>
       </c>
       <c r="B11" t="n">
-        <v>0.8533158439084443</v>
+        <v>0.7927984350132038</v>
       </c>
       <c r="C11" t="n">
-        <v>3.406267875490647</v>
+        <v>3.09691030480569</v>
       </c>
       <c r="D11" t="n">
-        <v>49.3560683249212</v>
+        <v>32.45699841927793</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>20904.6573</v>
+        <v>26103.4007</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -3151,64 +3151,64 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="J11" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="K11" t="n">
-        <v>19.49</v>
+        <v>15</v>
       </c>
       <c r="L11" t="n">
         <v>1500</v>
       </c>
       <c r="M11" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="N11" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="O11" t="n">
         <v>1.034</v>
       </c>
       <c r="P11" t="n">
-        <v>642.22253</v>
+        <v>701.938526</v>
       </c>
       <c r="Q11" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="R11" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="S11" t="n">
         <v>1.027</v>
       </c>
       <c r="T11" t="n">
-        <v>332.510351</v>
+        <v>361.314774</v>
       </c>
       <c r="U11" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="V11" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="W11" t="n">
         <v>1.02</v>
       </c>
       <c r="X11" t="n">
-        <v>200.694006</v>
+        <v>203.081721</v>
       </c>
       <c r="Y11" t="n">
-        <v>304.77259</v>
+        <v>273.469925</v>
       </c>
       <c r="Z11" t="n">
-        <v>10.8060298</v>
+        <v>9.70388799</v>
       </c>
       <c r="AA11" t="n">
         <v>1.034</v>
       </c>
       <c r="AB11" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AC11" t="n">
         <v>70</v>
@@ -3220,124 +3220,124 @@
         <v>50</v>
       </c>
       <c r="AF11" t="n">
-        <v>356.39105</v>
+        <v>442.372211</v>
       </c>
       <c r="AG11" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AH11" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AI11" t="n">
         <v>1.013</v>
       </c>
       <c r="AJ11" t="n">
-        <v>183.553063</v>
+        <v>188.776001</v>
       </c>
       <c r="AK11" t="n">
-        <v>357.1627</v>
+        <v>344.942565</v>
       </c>
       <c r="AL11" t="n">
-        <v>12.6635757</v>
+        <v>12.2400443</v>
       </c>
       <c r="AM11" t="n">
         <v>1.034</v>
       </c>
       <c r="AN11" t="n">
-        <v>593.7674929999999</v>
+        <v>640.143569</v>
       </c>
       <c r="AO11" t="n">
-        <v>-258041.636</v>
+        <v>-241187.022</v>
       </c>
       <c r="AP11" t="n">
-        <v>-40682.2538</v>
+        <v>-45346.1514</v>
       </c>
       <c r="AQ11" t="n">
-        <v>33.7663958</v>
+        <v>32.9836374</v>
       </c>
       <c r="AR11" t="n">
-        <v>393.073511</v>
+        <v>397.292713</v>
       </c>
       <c r="AS11" t="n">
-        <v>-298297.049</v>
+        <v>-286102.897</v>
       </c>
       <c r="AT11" t="n">
-        <v>52.3901092</v>
+        <v>71.4726392</v>
       </c>
       <c r="AU11" t="n">
-        <v>1.85754591</v>
+        <v>2.53615634</v>
       </c>
       <c r="AV11" t="n">
         <v>1.034</v>
       </c>
       <c r="AW11" t="n">
-        <v>642.222544</v>
+        <v>701.938525</v>
       </c>
       <c r="AX11" t="n">
-        <v>52.3901092</v>
+        <v>71.4726392</v>
       </c>
       <c r="AY11" t="n">
-        <v>1.85754591</v>
+        <v>2.53615634</v>
       </c>
       <c r="AZ11" t="n">
         <v>1.034</v>
       </c>
       <c r="BA11" t="n">
-        <v>300.370847</v>
+        <v>395.401446</v>
       </c>
       <c r="BB11" t="n">
-        <v>12.43752</v>
+        <v>8.17902602</v>
       </c>
       <c r="BC11" t="n">
-        <v>0.126670263</v>
+        <v>0.0832995141</v>
       </c>
       <c r="BD11" t="n">
-        <v>3.40626788</v>
+        <v>3.0969103</v>
       </c>
       <c r="BE11" t="n">
         <v>15</v>
       </c>
       <c r="BF11" t="n">
-        <v>12.43752</v>
+        <v>8.17902602</v>
       </c>
       <c r="BG11" t="n">
-        <v>0.126670263</v>
+        <v>0.0832995141</v>
       </c>
       <c r="BH11" t="n">
-        <v>3.40626788</v>
+        <v>3.0969103</v>
       </c>
       <c r="BI11" t="n">
-        <v>42.9338284</v>
+        <v>68.49652690000001</v>
       </c>
       <c r="BJ11" t="n">
-        <v>12.43752</v>
+        <v>8.17902602</v>
       </c>
       <c r="BK11" t="n">
-        <v>0.271624004</v>
+        <v>0.325981134</v>
       </c>
       <c r="BL11" t="n">
-        <v>3.40626788</v>
+        <v>3.0969103</v>
       </c>
       <c r="BM11" t="n">
-        <v>262.131444</v>
+        <v>341.011609</v>
       </c>
       <c r="BN11" t="n">
-        <v>0.288458853</v>
+        <v>0.00737969291</v>
       </c>
       <c r="BO11" t="n">
-        <v>0.533655861</v>
+        <v>0.74446523</v>
       </c>
       <c r="BP11" t="n">
-        <v>12.43752</v>
+        <v>8.17902602</v>
       </c>
       <c r="BQ11" t="n">
-        <v>0.271624004</v>
+        <v>0.325981134</v>
       </c>
       <c r="BR11" t="n">
-        <v>3.40626788</v>
+        <v>3.0969103</v>
       </c>
       <c r="BS11" t="n">
-        <v>283.358153</v>
+        <v>378.318</v>
       </c>
       <c r="BT11" t="n">
         <v>70</v>
@@ -3349,7 +3349,7 @@
         <v>50.07</v>
       </c>
       <c r="BW11" t="n">
-        <v>162.879568</v>
+        <v>172.363464</v>
       </c>
       <c r="BX11" t="n">
         <v>70</v>
@@ -3361,7 +3361,7 @@
         <v>50.05</v>
       </c>
       <c r="CA11" t="n">
-        <v>184.764796</v>
+        <v>189.948682</v>
       </c>
       <c r="CB11" t="n">
         <v>70</v>
@@ -3376,7 +3376,1277 @@
         <v>264.0032</v>
       </c>
       <c r="CF11" t="n">
-        <v>8.9</v>
+        <v>11.24</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>30</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.889260267313154</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2.119974806790662</v>
+      </c>
+      <c r="D12" t="n">
+        <v>35.8047784197648</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>18558.6009</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="J12" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="K12" t="n">
+        <v>15</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M12" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="N12" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="O12" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="P12" t="n">
+        <v>701.938526</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="R12" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="S12" t="n">
+        <v>1.027</v>
+      </c>
+      <c r="T12" t="n">
+        <v>380.650325</v>
+      </c>
+      <c r="U12" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="V12" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="W12" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="X12" t="n">
+        <v>204.272465</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>306.743717</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>10.8845851</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>701.938525</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>70</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>488.27746</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>1.013</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>190.370973</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>658.086542</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>-241187.022</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>-48078.1164</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>32.9836374</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>398.245854</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>-288833.909</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>38.1988474</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>1.35545924</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>701.938525</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>38.1988474</v>
+      </c>
+      <c r="AY12" t="n">
+        <v>1.35545924</v>
+      </c>
+      <c r="AZ12" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="BA12" t="n">
+        <v>288.979328</v>
+      </c>
+      <c r="BB12" t="n">
+        <v>9.022652389999999</v>
+      </c>
+      <c r="BC12" t="n">
+        <v>0.09189144990000001</v>
+      </c>
+      <c r="BD12" t="n">
+        <v>2.11997481</v>
+      </c>
+      <c r="BE12" t="n">
+        <v>15</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>9.022652389999999</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>0.09189144990000001</v>
+      </c>
+      <c r="BH12" t="n">
+        <v>2.11997481</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>51.5029919</v>
+      </c>
+      <c r="BJ12" t="n">
+        <v>9.022652389999999</v>
+      </c>
+      <c r="BK12" t="n">
+        <v>0.247491616</v>
+      </c>
+      <c r="BL12" t="n">
+        <v>2.11997481</v>
+      </c>
+      <c r="BM12" t="n">
+        <v>253.076982</v>
+      </c>
+      <c r="BN12" t="n">
+        <v>0.161721551</v>
+      </c>
+      <c r="BO12" t="n">
+        <v>0.628708837</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>9.022652389999999</v>
+      </c>
+      <c r="BQ12" t="n">
+        <v>0.247491616</v>
+      </c>
+      <c r="BR12" t="n">
+        <v>2.11997481</v>
+      </c>
+      <c r="BS12" t="n">
+        <v>280.911347</v>
+      </c>
+      <c r="BT12" t="n">
+        <v>70</v>
+      </c>
+      <c r="BU12" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="BV12" t="n">
+        <v>50.07</v>
+      </c>
+      <c r="BW12" t="n">
+        <v>174.42197</v>
+      </c>
+      <c r="BX12" t="n">
+        <v>70</v>
+      </c>
+      <c r="BY12" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="BZ12" t="n">
+        <v>50.05</v>
+      </c>
+      <c r="CA12" t="n">
+        <v>191.496604</v>
+      </c>
+      <c r="CB12" t="n">
+        <v>70</v>
+      </c>
+      <c r="CC12" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="CD12" t="n">
+        <v>50.05</v>
+      </c>
+      <c r="CE12" t="n">
+        <v>264.0032</v>
+      </c>
+      <c r="CF12" t="n">
+        <v>10.6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>60</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.9087561447269246</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4.555764628576739</v>
+      </c>
+      <c r="D13" t="n">
+        <v>39.56547202740087</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>15283.6297</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="J13" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="K13" t="n">
+        <v>15</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M13" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="N13" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="O13" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="P13" t="n">
+        <v>701.938526</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="R13" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="S13" t="n">
+        <v>1.027</v>
+      </c>
+      <c r="T13" t="n">
+        <v>389.834614</v>
+      </c>
+      <c r="U13" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="V13" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="W13" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="X13" t="n">
+        <v>204.921171</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>313.468675</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>11.1232155</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>701.938525</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>70</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>508.241638</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>1.013</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>191.136262</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>665.853826</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>-241187.022</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>-49271.9219</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>32.9836374</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>398.660882</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>-290027.299</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>31.4738894</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>1.11682883</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>701.938525</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>31.4738894</v>
+      </c>
+      <c r="AY13" t="n">
+        <v>1.11682883</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>289.19813</v>
+      </c>
+      <c r="BB13" t="n">
+        <v>9.97033124</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>0.101543111</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>4.55576463</v>
+      </c>
+      <c r="BE13" t="n">
+        <v>15</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>9.97033124</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>0.101543111</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>4.55576463</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>49.1926841</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>9.97033124</v>
+      </c>
+      <c r="BK13" t="n">
+        <v>0.197837722</v>
+      </c>
+      <c r="BL13" t="n">
+        <v>4.55576463</v>
+      </c>
+      <c r="BM13" t="n">
+        <v>260.147254</v>
+      </c>
+      <c r="BN13" t="n">
+        <v>0.351019547</v>
+      </c>
+      <c r="BO13" t="n">
+        <v>0.48673534</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>9.97033124</v>
+      </c>
+      <c r="BQ13" t="n">
+        <v>0.197837722</v>
+      </c>
+      <c r="BR13" t="n">
+        <v>4.55576463</v>
+      </c>
+      <c r="BS13" t="n">
+        <v>286.465498</v>
+      </c>
+      <c r="BT13" t="n">
+        <v>70</v>
+      </c>
+      <c r="BU13" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="BV13" t="n">
+        <v>50.07</v>
+      </c>
+      <c r="BW13" t="n">
+        <v>175.309098</v>
+      </c>
+      <c r="BX13" t="n">
+        <v>70</v>
+      </c>
+      <c r="BY13" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="BZ13" t="n">
+        <v>50.05</v>
+      </c>
+      <c r="CA13" t="n">
+        <v>192.246657</v>
+      </c>
+      <c r="CB13" t="n">
+        <v>70</v>
+      </c>
+      <c r="CC13" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="CD13" t="n">
+        <v>50.05</v>
+      </c>
+      <c r="CE13" t="n">
+        <v>264.0032</v>
+      </c>
+      <c r="CF13" t="n">
+        <v>10.27</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>57</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.8684156618597763</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1.915986273500752</v>
+      </c>
+      <c r="D14" t="n">
+        <v>43.06757937310909</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>21896.9036</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="J14" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="K14" t="n">
+        <v>15</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M14" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="N14" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="O14" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="P14" t="n">
+        <v>701.938526</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="R14" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="S14" t="n">
+        <v>1.027</v>
+      </c>
+      <c r="T14" t="n">
+        <v>371.787927</v>
+      </c>
+      <c r="U14" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="V14" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="W14" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="X14" t="n">
+        <v>203.693386</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>299.553525</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>10.6294462</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>701.938525</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>70</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>467.924478</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>1.013</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>189.636698</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>650.155857</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>-241187.022</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>-46865.3443</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>32.9836374</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>397.823492</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>-287621.559</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>45.389039</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>1.61059813</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AW14" t="n">
+        <v>701.938525</v>
+      </c>
+      <c r="AX14" t="n">
+        <v>45.389039</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>1.61059813</v>
+      </c>
+      <c r="AZ14" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>292.030419</v>
+      </c>
+      <c r="BB14" t="n">
+        <v>10.8528474</v>
+      </c>
+      <c r="BC14" t="n">
+        <v>0.110531122</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>1.91598627</v>
+      </c>
+      <c r="BE14" t="n">
+        <v>15</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>10.8528474</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>0.110531122</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>1.91598627</v>
+      </c>
+      <c r="BI14" t="n">
+        <v>45.6843605</v>
+      </c>
+      <c r="BJ14" t="n">
+        <v>10.8528474</v>
+      </c>
+      <c r="BK14" t="n">
+        <v>0.291678817</v>
+      </c>
+      <c r="BL14" t="n">
+        <v>1.91598627</v>
+      </c>
+      <c r="BM14" t="n">
+        <v>253.199304</v>
+      </c>
+      <c r="BN14" t="n">
+        <v>0.171930746</v>
+      </c>
+      <c r="BO14" t="n">
+        <v>0.6210519410000001</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>10.8528474</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>0.291678817</v>
+      </c>
+      <c r="BR14" t="n">
+        <v>1.91598627</v>
+      </c>
+      <c r="BS14" t="n">
+        <v>276.513237</v>
+      </c>
+      <c r="BT14" t="n">
+        <v>70</v>
+      </c>
+      <c r="BU14" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="BV14" t="n">
+        <v>50.07</v>
+      </c>
+      <c r="BW14" t="n">
+        <v>173.513453</v>
+      </c>
+      <c r="BX14" t="n">
+        <v>70</v>
+      </c>
+      <c r="BY14" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="BZ14" t="n">
+        <v>50.05</v>
+      </c>
+      <c r="CA14" t="n">
+        <v>190.781088</v>
+      </c>
+      <c r="CB14" t="n">
+        <v>70</v>
+      </c>
+      <c r="CC14" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="CD14" t="n">
+        <v>50.05</v>
+      </c>
+      <c r="CE14" t="n">
+        <v>264.0032</v>
+      </c>
+      <c r="CF14" t="n">
+        <v>11.26</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>43</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.9276593047170996</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2.198678647321549</v>
+      </c>
+      <c r="D15" t="n">
+        <v>46.12936144555182</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>13359.2936</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="J15" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="K15" t="n">
+        <v>15</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M15" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="N15" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="P15" t="n">
+        <v>701.938526</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="R15" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="S15" t="n">
+        <v>1.027</v>
+      </c>
+      <c r="T15" t="n">
+        <v>395.46827</v>
+      </c>
+      <c r="U15" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="V15" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="W15" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="X15" t="n">
+        <v>205.33455</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>319.98918</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>11.354591</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>701.938525</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>70</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>519.962983</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>1.013</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>191.601153</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>670.411968</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>-241187.022</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>-49975.2987</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>32.9836374</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>398.905207</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>-290730.432</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>24.9533849</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>0.885453317</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>701.938525</v>
+      </c>
+      <c r="AX15" t="n">
+        <v>24.9533849</v>
+      </c>
+      <c r="AY15" t="n">
+        <v>0.885453317</v>
+      </c>
+      <c r="AZ15" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>244.473229</v>
+      </c>
+      <c r="BB15" t="n">
+        <v>11.6244035</v>
+      </c>
+      <c r="BC15" t="n">
+        <v>0.118389056</v>
+      </c>
+      <c r="BD15" t="n">
+        <v>2.19867865</v>
+      </c>
+      <c r="BE15" t="n">
+        <v>15</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>11.6244035</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>0.118389056</v>
+      </c>
+      <c r="BH15" t="n">
+        <v>2.19867865</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>40.2992502</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>11.6244035</v>
+      </c>
+      <c r="BK15" t="n">
+        <v>0.183161964</v>
+      </c>
+      <c r="BL15" t="n">
+        <v>2.19867865</v>
+      </c>
+      <c r="BM15" t="n">
+        <v>222.976662</v>
+      </c>
+      <c r="BN15" t="n">
+        <v>0.528483558</v>
+      </c>
+      <c r="BO15" t="n">
+        <v>0.353637331</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>11.6244035</v>
+      </c>
+      <c r="BQ15" t="n">
+        <v>0.183161964</v>
+      </c>
+      <c r="BR15" t="n">
+        <v>2.19867865</v>
+      </c>
+      <c r="BS15" t="n">
+        <v>243.658175</v>
+      </c>
+      <c r="BT15" t="n">
+        <v>70</v>
+      </c>
+      <c r="BU15" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="BV15" t="n">
+        <v>50.07</v>
+      </c>
+      <c r="BW15" t="n">
+        <v>175.828769</v>
+      </c>
+      <c r="BX15" t="n">
+        <v>70</v>
+      </c>
+      <c r="BY15" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="BZ15" t="n">
+        <v>50.05</v>
+      </c>
+      <c r="CA15" t="n">
+        <v>192.703818</v>
+      </c>
+      <c r="CB15" t="n">
+        <v>70</v>
+      </c>
+      <c r="CC15" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="CD15" t="n">
+        <v>50.05</v>
+      </c>
+      <c r="CE15" t="n">
+        <v>264.0032</v>
+      </c>
+      <c r="CF15" t="n">
+        <v>11.66</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>78</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.8120216641557021</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1.813047790211846</v>
+      </c>
+      <c r="D16" t="n">
+        <v>49.64585859029136</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>28794.4095</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="J16" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="K16" t="n">
+        <v>15</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M16" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="N16" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="O16" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="P16" t="n">
+        <v>701.938526</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="R16" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="S16" t="n">
+        <v>1.027</v>
+      </c>
+      <c r="T16" t="n">
+        <v>355.0111</v>
+      </c>
+      <c r="U16" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="V16" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="W16" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="X16" t="n">
+        <v>202.757287</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>280.100835</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>9.939181169999999</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>701.938525</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>70</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>426.123387</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>1.013</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>188.259666</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>344.942565</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>12.2400443</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>633.727157</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>-241187.022</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>-44380.0643</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>32.9836374</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>396.953765</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>-285137.149</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>64.8417292</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>2.30086316</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>701.938525</v>
+      </c>
+      <c r="AX16" t="n">
+        <v>64.8417292</v>
+      </c>
+      <c r="AY16" t="n">
+        <v>2.30086316</v>
+      </c>
+      <c r="AZ16" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="BA16" t="n">
+        <v>326.147634</v>
+      </c>
+      <c r="BB16" t="n">
+        <v>12.5105459</v>
+      </c>
+      <c r="BC16" t="n">
+        <v>0.127413997</v>
+      </c>
+      <c r="BD16" t="n">
+        <v>1.81304779</v>
+      </c>
+      <c r="BE16" t="n">
+        <v>15</v>
+      </c>
+      <c r="BF16" t="n">
+        <v>12.5105459</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>0.127413997</v>
+      </c>
+      <c r="BH16" t="n">
+        <v>1.81304779</v>
+      </c>
+      <c r="BI16" t="n">
+        <v>42.8710288</v>
+      </c>
+      <c r="BJ16" t="n">
+        <v>12.5105459</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>0.380980654</v>
+      </c>
+      <c r="BL16" t="n">
+        <v>1.81304779</v>
+      </c>
+      <c r="BM16" t="n">
+        <v>263.915015</v>
+      </c>
+      <c r="BN16" t="n">
+        <v>0.112582562</v>
+      </c>
+      <c r="BO16" t="n">
+        <v>0.665563079</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>12.5105459</v>
+      </c>
+      <c r="BQ16" t="n">
+        <v>0.380980654</v>
+      </c>
+      <c r="BR16" t="n">
+        <v>1.81304779</v>
+      </c>
+      <c r="BS16" t="n">
+        <v>284.583925</v>
+      </c>
+      <c r="BT16" t="n">
+        <v>70</v>
+      </c>
+      <c r="BU16" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="BV16" t="n">
+        <v>50.07</v>
+      </c>
+      <c r="BW16" t="n">
+        <v>171.624227</v>
+      </c>
+      <c r="BX16" t="n">
+        <v>70</v>
+      </c>
+      <c r="BY16" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="BZ16" t="n">
+        <v>50.05</v>
+      </c>
+      <c r="CA16" t="n">
+        <v>189.453142</v>
+      </c>
+      <c r="CB16" t="n">
+        <v>70</v>
+      </c>
+      <c r="CC16" t="n">
+        <v>3.88559045</v>
+      </c>
+      <c r="CD16" t="n">
+        <v>50.05</v>
+      </c>
+      <c r="CE16" t="n">
+        <v>264.0032</v>
+      </c>
+      <c r="CF16" t="n">
+        <v>9.470000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -3424,7 +4694,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -3434,7 +4704,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>79</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5">

</xml_diff>